<commit_message>
update short ins-nia & invariant & binding 66a8bdff77990c2cb2beba5a65da5fe5ee982f14
</commit_message>
<xml_diff>
--- a/nr-update-patient-identifiers/ig/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/nr-update-patient-identifiers/ig/StructureDefinition-fr-core-patient-ins.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-07-15T08:52:52+00:00</t>
+    <t>2025-07-17T15:24:19+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -279,7 +279,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}fr-core-1:If identityReliability status = 'VALI', then at least Patient.identifier[INS-NIR] or Patient.identifier[INS-NIA] or Patient.identifier[INS-NIR-TEST]or Patient.identifier[INS-NIR-DEMO] SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.8' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.9' and use = 'temp').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.10' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.11' and use = 'official').exists())}fr-core-2:If identityReliability status = 'VALI', then only one identifier of type official SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(use = 'official').count() = 1 or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.9' and use = 'temp').exists())}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}fr-core-1:If identityReliability status = 'VALI', then at least Patient.identifier[INS-NIR] or Patient.identifier[INS-NIA] or Patient.identifier[INS-NIR-TEST]or Patient.identifier[INS-NIR-DEMO] SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.8' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.9' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.10' and use = 'official').exists() or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.11' and use = 'official').exists())}fr-core-2:If identityReliability status = 'VALI', then only one identifier of type official SHALL be present {(extension('https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-identity-reliability').extension('identityStatus').value.exists(code = 'VALI')) implies (identifier.where(use = 'official').count() = 1 or identifier.where(system = 'urn:oid:1.2.250.1.213.1.4.9' and use = 'temp').exists())}</t>
   </si>
   <si>
     <t>Patient[classCode=PAT]</t>
@@ -1579,6 +1579,9 @@
     <t>Patient.identifier:INS-NIR.use</t>
   </si>
   <si>
+    <t>official | old</t>
+  </si>
+  <si>
     <t>La valeur old permet d'identifier des INS désactivés (permettant de noter l'ancien INS-NIR en cas de changement de sexe par exemple)</t>
   </si>
   <si>
@@ -1730,9 +1733,6 @@
   </si>
   <si>
     <t>La valeur old permet d'identifier des INS désactivés (en cas d'obtention d'un INS-NIR par exemple)</t>
-  </si>
-  <si>
-    <t>temp</t>
   </si>
   <si>
     <t>Patient.identifier:INS-NIA.type</t>
@@ -13885,13 +13885,13 @@
         <v>172</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>379</v>
+        <v>494</v>
       </c>
       <c r="M93" t="s" s="2">
         <v>380</v>
       </c>
       <c r="N93" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="O93" t="s" s="2">
         <v>382</v>
@@ -13923,7 +13923,7 @@
       </c>
       <c r="Y93" s="2"/>
       <c r="Z93" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="AA93" t="s" s="2">
         <v>82</v>
@@ -13973,7 +13973,7 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B94" t="s" s="2">
         <v>389</v>
@@ -14021,7 +14021,7 @@
         <v>82</v>
       </c>
       <c r="S94" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="T94" t="s" s="2">
         <v>82</v>
@@ -14039,10 +14039,10 @@
         <v>154</v>
       </c>
       <c r="Y94" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="Z94" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="AA94" t="s" s="2">
         <v>82</v>
@@ -14092,7 +14092,7 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B95" t="s" s="2">
         <v>400</v>
@@ -14121,7 +14121,7 @@
         <v>132</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="M95" t="s" s="2">
         <v>402</v>
@@ -14211,7 +14211,7 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B96" t="s" s="2">
         <v>411</v>
@@ -14328,7 +14328,7 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B97" t="s" s="2">
         <v>420</v>
@@ -14443,7 +14443,7 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B98" t="s" s="2">
         <v>427</v>
@@ -14560,13 +14560,13 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B99" t="s" s="2">
         <v>359</v>
       </c>
       <c r="C99" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D99" t="s" s="2">
         <v>82</v>
@@ -14591,7 +14591,7 @@
         <v>360</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="M99" t="s" s="2">
         <v>362</v>
@@ -14679,7 +14679,7 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B100" t="s" s="2">
         <v>374</v>
@@ -14794,7 +14794,7 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B101" t="s" s="2">
         <v>376</v>
@@ -14911,7 +14911,7 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B102" t="s" s="2">
         <v>378</v>
@@ -15030,7 +15030,7 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B103" t="s" s="2">
         <v>389</v>
@@ -15078,7 +15078,7 @@
         <v>82</v>
       </c>
       <c r="S103" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="T103" t="s" s="2">
         <v>82</v>
@@ -15096,10 +15096,10 @@
         <v>154</v>
       </c>
       <c r="Y103" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="Z103" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="AA103" t="s" s="2">
         <v>82</v>
@@ -15149,7 +15149,7 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B104" t="s" s="2">
         <v>400</v>
@@ -15178,7 +15178,7 @@
         <v>132</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="M104" t="s" s="2">
         <v>402</v>
@@ -15197,7 +15197,7 @@
         <v>82</v>
       </c>
       <c r="S104" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="T104" t="s" s="2">
         <v>406</v>
@@ -15268,7 +15268,7 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B105" t="s" s="2">
         <v>411</v>
@@ -15385,7 +15385,7 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B106" t="s" s="2">
         <v>420</v>
@@ -15500,7 +15500,7 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B107" t="s" s="2">
         <v>427</v>
@@ -15617,13 +15617,13 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B108" t="s" s="2">
         <v>359</v>
       </c>
       <c r="C108" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D108" t="s" s="2">
         <v>82</v>
@@ -15648,7 +15648,7 @@
         <v>360</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="M108" t="s" s="2">
         <v>362</v>
@@ -15736,7 +15736,7 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B109" t="s" s="2">
         <v>374</v>
@@ -15851,7 +15851,7 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B110" t="s" s="2">
         <v>376</v>
@@ -15968,7 +15968,7 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B111" t="s" s="2">
         <v>378</v>
@@ -16087,7 +16087,7 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B112" t="s" s="2">
         <v>389</v>
@@ -16135,7 +16135,7 @@
         <v>82</v>
       </c>
       <c r="S112" t="s" s="2">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="T112" t="s" s="2">
         <v>82</v>
@@ -16153,10 +16153,10 @@
         <v>154</v>
       </c>
       <c r="Y112" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="Z112" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="AA112" t="s" s="2">
         <v>82</v>
@@ -16206,7 +16206,7 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B113" t="s" s="2">
         <v>400</v>
@@ -16235,7 +16235,7 @@
         <v>132</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="M113" t="s" s="2">
         <v>402</v>
@@ -16254,7 +16254,7 @@
         <v>82</v>
       </c>
       <c r="S113" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="T113" t="s" s="2">
         <v>406</v>
@@ -16325,7 +16325,7 @@
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B114" t="s" s="2">
         <v>411</v>
@@ -16442,7 +16442,7 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B115" t="s" s="2">
         <v>420</v>
@@ -16557,7 +16557,7 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B116" t="s" s="2">
         <v>427</v>
@@ -16674,13 +16674,13 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B117" t="s" s="2">
         <v>359</v>
       </c>
       <c r="C117" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="D117" t="s" s="2">
         <v>82</v>
@@ -16705,7 +16705,7 @@
         <v>360</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="M117" t="s" s="2">
         <v>362</v>
@@ -16793,7 +16793,7 @@
     </row>
     <row r="118" hidden="true">
       <c r="A118" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B118" t="s" s="2">
         <v>374</v>
@@ -16908,7 +16908,7 @@
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B119" t="s" s="2">
         <v>376</v>
@@ -17025,7 +17025,7 @@
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B120" t="s" s="2">
         <v>378</v>
@@ -17054,13 +17054,13 @@
         <v>172</v>
       </c>
       <c r="L120" t="s" s="2">
-        <v>379</v>
+        <v>494</v>
       </c>
       <c r="M120" t="s" s="2">
         <v>380</v>
       </c>
       <c r="N120" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="O120" t="s" s="2">
         <v>382</v>
@@ -17073,7 +17073,7 @@
         <v>82</v>
       </c>
       <c r="S120" t="s" s="2">
-        <v>540</v>
+        <v>82</v>
       </c>
       <c r="T120" t="s" s="2">
         <v>82</v>
@@ -17092,7 +17092,7 @@
       </c>
       <c r="Y120" s="2"/>
       <c r="Z120" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="AA120" t="s" s="2">
         <v>82</v>
@@ -17208,10 +17208,10 @@
         <v>154</v>
       </c>
       <c r="Y121" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="Z121" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="AA121" t="s" s="2">
         <v>82</v>

</xml_diff>